<commit_message>
updated 4.0 m odel
</commit_message>
<xml_diff>
--- a/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
+++ b/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\RMI-temp\bldgs\SYDEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\bldgs\SYDEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D978AB-7610-4385-B33B-1C4B4735BABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F68715-1BDC-4F96-B4F9-DAECB448B85E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="14910" windowHeight="14820" tabRatio="670" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="670" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -2252,9 +2252,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="15"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -2275,6 +2272,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="10">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="16">
@@ -29232,43 +29232,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>419</v>
       </c>
-      <c r="B1" s="30"/>
+      <c r="B1" s="29"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="30" t="s">
         <v>418</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
     </row>
     <row r="3" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="27"/>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="34"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="33"/>
     </row>
     <row r="4" spans="1:7" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="27"/>
       <c r="B4" s="26"/>
-      <c r="C4" s="35" t="s">
+      <c r="C4" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="34"/>
     </row>
     <row r="5" spans="1:7" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25"/>
@@ -34209,15 +34209,15 @@
       <c r="G220" s="11"/>
     </row>
     <row r="221" spans="1:7" s="4" customFormat="1" ht="206.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A221" s="36" t="s">
+      <c r="A221" s="35" t="s">
         <v>393</v>
       </c>
-      <c r="B221" s="36"/>
-      <c r="C221" s="36"/>
-      <c r="D221" s="36"/>
-      <c r="E221" s="36"/>
-      <c r="F221" s="36"/>
-      <c r="G221" s="36"/>
+      <c r="B221" s="35"/>
+      <c r="C221" s="35"/>
+      <c r="D221" s="35"/>
+      <c r="E221" s="35"/>
+      <c r="F221" s="35"/>
+      <c r="G221" s="35"/>
     </row>
     <row r="222" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222"/>
@@ -34298,13 +34298,16 @@
         <v>546</v>
       </c>
       <c r="B4">
+        <f>INDEX('AEO Table 21'!$E$77:$AK$77,MATCH(About!$A$22,'AEO Table 21'!$E$5:$AK$5,0))*GW_to_MW*About!$A$25</f>
         <v>0</v>
       </c>
       <c r="C4">
+        <f>INDEX('AEO Table 21'!$E$77:$AK$77,MATCH(About!$A$22,'AEO Table 21'!$E$5:$AK$5,0))*GW_to_MW*About!$A$25</f>
         <v>0</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <f>INDEX('AEO Table 22'!$E$60:$AK$60,MATCH(About!$A$22,'AEO Table 22'!$E$5:$AK$5,0))*GW_to_MW</f>
+        <v>1377.152</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -34340,13 +34343,16 @@
         <v>59</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <f>INDEX('AEO Table 21'!$E$79:$AK$79,MATCH(About!$A$22,'AEO Table 21'!$E$5:$AK$5,0))*GW_to_MW*About!$A$25</f>
+        <v>11.571780781996274</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <f>INDEX('AEO Table 21'!$E$79:$AK$79,MATCH(About!$A$22,'AEO Table 21'!$E$5:$AK$5,0))*GW_to_MW*About!$A$26</f>
+        <v>2.6602192180037236</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <f>INDEX('AEO Table 22'!$E$62:$AK$62,MATCH(About!$A$22,'AEO Table 22'!$E$5:$AK$5,0))*GW_to_MW</f>
+        <v>554.88099999999997</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -34354,13 +34360,16 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <f>INDEX('AEO Table 21'!$E$78:$AK$78,MATCH(About!$A$22,'AEO Table 21'!$E$5:$AK$5,0))*GW_to_MW*About!$A$25</f>
+        <v>14894.199872095845</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <f>INDEX('AEO Table 21'!$E$78:$AK$78,MATCH(About!$A$22,'AEO Table 21'!$E$5:$AK$5,0))*GW_to_MW*About!$A$26</f>
+        <v>3424.0051279041522</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <f>INDEX('AEO Table 22'!$E$61:$AK$61,MATCH(About!$A$22,'AEO Table 22'!$E$5:$AK$5,0))*GW_to_MW</f>
+        <v>15855.377</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -34416,7 +34425,8 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <f>INDEX('AEO Table 22'!$E$59:$AK$59,MATCH(About!$A$22,'AEO Table 22'!$E$5:$AK$5,0))*GW_to_MW</f>
+        <v>17.117000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -34574,7 +34584,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="36" t="s">
         <v>552</v>
       </c>
       <c r="B24">
@@ -34588,7 +34598,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="36" t="s">
         <v>553</v>
       </c>
       <c r="B25">

</xml_diff>